<commit_message>
feat: add offline report tracking and run comparison
Complete T-507, T-508 and T-602 with restricted tracking projections, qualified comparisons, deterministic snapshot bindings and synthetic acceptance.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: 9c7fa8f8-60e8-4888-9220-dca7558312eb
</commit_message>
<xml_diff>
--- a/template/ApimActionPlan.xlsx
+++ b/template/ApimActionPlan.xlsx
@@ -16,14 +16,20 @@
     <sheet name="Cost" sheetId="9" r:id="rId10"/>
     <sheet name="Environment Drift" sheetId="10" r:id="rId11"/>
     <sheet name="Run Info" sheetId="11" r:id="rId12"/>
-    <sheet name="Method &amp; Rules" sheetId="12" r:id="rId13"/>
+    <sheet name="Resolved Since Last Run" sheetId="12" r:id="rId13"/>
+    <sheet name="Not Reassessed" sheetId="13" r:id="rId14"/>
+    <sheet name="Run Comparison" sheetId="14" r:id="rId15"/>
+    <sheet name="Comparison Gaps" sheetId="15" r:id="rId16"/>
+    <sheet name="Comparison Pillars" sheetId="16" r:id="rId17"/>
+    <sheet name="Comparison KPIs" sheetId="17" r:id="rId18"/>
+    <sheet name="Method &amp; Rules" sheetId="18" r:id="rId19"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="194">
   <si>
     <t>APIM Assessment Summary</t>
   </si>
@@ -514,6 +520,81 @@
     <t>Value</t>
   </si>
   <si>
+    <t>Resolved Since Last Run</t>
+  </si>
+  <si>
+    <t>Absent from comparable evaluated results; not proof of remediation</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Change</t>
+  </si>
+  <si>
+    <t>Not Reassessed</t>
+  </si>
+  <si>
+    <t>Prior tracking retained where current evidence cannot establish resolution</t>
+  </si>
+  <si>
+    <t>Run Comparison</t>
+  </si>
+  <si>
+    <t>Comparable evaluated snapshots; absence is not independently verified remediation</t>
+  </si>
+  <si>
+    <t>Previous Severity</t>
+  </si>
+  <si>
+    <t>Current Severity</t>
+  </si>
+  <si>
+    <t>Severity Changed</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Comparison Data Gaps</t>
+  </si>
+  <si>
+    <t>Unavailable or changed assessment coverage is not a resolved finding</t>
+  </si>
+  <si>
+    <t>Comparison by Pillar</t>
+  </si>
+  <si>
+    <t>Counts of comparable changes and not-reassessed rows</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>Persisting</t>
+  </si>
+  <si>
+    <t>Comparison KPIs</t>
+  </si>
+  <si>
+    <t>Unavailable values and deltas remain blank with explicit reasons</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Baseline</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
     <t>Method &amp; Rules</t>
   </si>
   <si>
@@ -924,7 +1005,103 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblRules" displayName="tblRules" ref="A3:J4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblResolvedTracking" displayName="tblResolvedTracking" ref="A3:H4" headerRowCount="1">
+  <autoFilter ref="A3:H4"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Kind"/>
+    <tableColumn id="2" name="Key"/>
+    <tableColumn id="3" name="Rule ID"/>
+    <tableColumn id="4" name="Change"/>
+    <tableColumn id="5" name="Owner"/>
+    <tableColumn id="6" name="Status"/>
+    <tableColumn id="7" name="Target Date"/>
+    <tableColumn id="8" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblUnassessedTracking" displayName="tblUnassessedTracking" ref="A3:H4" headerRowCount="1">
+  <autoFilter ref="A3:H4"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Kind"/>
+    <tableColumn id="2" name="Key"/>
+    <tableColumn id="3" name="Rule ID"/>
+    <tableColumn id="4" name="Change"/>
+    <tableColumn id="5" name="Owner"/>
+    <tableColumn id="6" name="Status"/>
+    <tableColumn id="7" name="Target Date"/>
+    <tableColumn id="8" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblComparison" displayName="tblComparison" ref="A3:H4" headerRowCount="1">
+  <autoFilter ref="A3:H4"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Finding Key"/>
+    <tableColumn id="2" name="Rule ID"/>
+    <tableColumn id="3" name="Pillar"/>
+    <tableColumn id="4" name="Change"/>
+    <tableColumn id="5" name="Previous Severity"/>
+    <tableColumn id="6" name="Current Severity"/>
+    <tableColumn id="7" name="Severity Changed"/>
+    <tableColumn id="8" name="Reason"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblComparisonGaps" displayName="tblComparisonGaps" ref="A3:H4" headerRowCount="1">
+  <autoFilter ref="A3:H4"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Finding Key"/>
+    <tableColumn id="2" name="Rule ID"/>
+    <tableColumn id="3" name="Pillar"/>
+    <tableColumn id="4" name="Change"/>
+    <tableColumn id="5" name="Previous Severity"/>
+    <tableColumn id="6" name="Current Severity"/>
+    <tableColumn id="7" name="Severity Changed"/>
+    <tableColumn id="8" name="Reason"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblComparisonPillars" displayName="tblComparisonPillars" ref="A3:E4" headerRowCount="1">
+  <autoFilter ref="A3:E4"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Pillar"/>
+    <tableColumn id="2" name="New"/>
+    <tableColumn id="3" name="Resolved"/>
+    <tableColumn id="4" name="Persisting"/>
+    <tableColumn id="5" name="Not Reassessed"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblComparisonKpis" displayName="tblComparisonKpis" ref="A3:E4" headerRowCount="1">
+  <autoFilter ref="A3:E4"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Metric"/>
+    <tableColumn id="2" name="Baseline"/>
+    <tableColumn id="3" name="Current"/>
+    <tableColumn id="4" name="Delta"/>
+    <tableColumn id="5" name="Reason"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblRules" displayName="tblRules" ref="A3:J4" headerRowCount="1">
   <autoFilter ref="A3:J4"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Rule ID"/>
@@ -942,8 +1119,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblWeights" displayName="tblWeights" ref="M3:O4" headerRowCount="1">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblWeights" displayName="tblWeights" ref="M3:O4" headerRowCount="1">
   <autoFilter ref="M3:O4"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Dimension"/>
@@ -1663,6 +1840,438 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4"/>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4"/>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4"/>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4"/>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4"/>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4"/>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:O10000"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1683,7 +2292,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="13" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -1702,7 +2311,7 @@
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="14" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -1739,7 +2348,7 @@
         <v>38</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="H3" s="0" t="s">
         <v>28</v>
@@ -1748,16 +2357,16 @@
         <v>29</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="M3" s="0" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
       <c r="N3" s="0" t="s">
         <v>162</v>
       </c>
       <c r="O3" s="0" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4">
@@ -92051,6 +92660,11 @@
       <formula>NOT(ISERROR(SEARCH("Info",F4)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="S4:S10000" showErrorMessage="1" errorTitle="Invalid status" error="Select a status from the list.">
+      <formula1>"Open,In progress,Done,Accepted risk,Not applicable"</formula1>
+    </dataValidation>
+  </dataValidations>
   <headerFooter/>
   <tableParts>
     <tablePart r:id="rId1"/>

</xml_diff>